<commit_message>
Transfer: botón Transfer en lugar de Excel, Imprimir Transfer para plantilla
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/templates/PLANTILLA TRANSFER DIRECTO CRM.xlsx
+++ b/templates/PLANTILLA TRANSFER DIRECTO CRM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pacol\CURSOR\CRM_Gemavip\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB27970E-8784-4246-8D93-B72BA8F86CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5882DD-1AA2-4917-882C-7C79A04F5431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{43D4710E-17FA-46CC-9775-DF7A3B84A70C}"/>
   </bookViews>
@@ -441,13 +441,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -865,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22833EA7-2433-4E1A-8046-D61A0D7088BE}">
-  <dimension ref="B3:F34"/>
+  <dimension ref="B3:F45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.375" defaultRowHeight="12.9" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.375" style="2" customWidth="1"/>
@@ -1325,10 +1325,10 @@
     </row>
     <row r="4" spans="2:6" ht="13.6" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="33"/>
+      <c r="C5" s="34"/>
       <c r="D5" s="4" t="s">
         <v>2</v>
       </c>
@@ -1524,20 +1524,97 @@
       <c r="F27" s="25"/>
     </row>
     <row r="28" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
-      <c r="B28" s="34" t="s">
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="25"/>
+    </row>
+    <row r="29" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="25"/>
+    </row>
+    <row r="30" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="25"/>
+    </row>
+    <row r="31" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="25"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="25"/>
+    </row>
+    <row r="33" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="25"/>
+    </row>
+    <row r="34" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="25"/>
+    </row>
+    <row r="35" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="25"/>
+    </row>
+    <row r="36" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="25"/>
+    </row>
+    <row r="37" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B37" s="25"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="25"/>
+    </row>
+    <row r="38" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B38" s="25"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="25"/>
+    </row>
+    <row r="39" spans="2:6" ht="15.65" x14ac:dyDescent="0.25">
+      <c r="B39" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="32" spans="2:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" spans="6:6" ht="27.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" spans="6:6" ht="27.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F34" s="2"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="43" spans="2:6" ht="15.65" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="2:6" ht="27.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" spans="2:6" ht="27.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F45" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>